<commit_message>
feat: added name table to every sheet in the excel
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Laptop\e\VVSS\CamiVVSS_ro2025-2026\Labs\CheckListsAll\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moglan Calin-Stefan\CS UBB\SEM6\VVSS\MyDrinkShop\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE83867-3721-469D-B0A3-67FDA22FF09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F88C50A-6EA3-4AE1-AA21-0C13316182AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2940" yWindow="3255" windowWidth="38700" windowHeight="15825" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="35">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Reviewer Name:</t>
   </si>
   <si>
-    <t>do not print this form</t>
-  </si>
-  <si>
     <t>Crt. No.</t>
   </si>
   <si>
@@ -77,9 +74,6 @@
     <t>Georgescu Anca</t>
   </si>
   <si>
-    <t>Firicescu George</t>
-  </si>
-  <si>
     <t>Requirements Document</t>
   </si>
   <si>
@@ -135,19 +129,38 @@
   </si>
   <si>
     <t>Effort to perform tool-based code analysis (hours):</t>
+  </si>
+  <si>
+    <t>Moglan Calin-Stefan</t>
+  </si>
+  <si>
+    <t>Valentin Munteanu</t>
+  </si>
+  <si>
+    <t>Moise Ioana</t>
+  </si>
+  <si>
+    <t>Munteanu Valentin-Ioan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -326,79 +339,80 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,109 +721,122 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.26953125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="21" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.90625" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="4" width="16.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="7" width="8.85546875" style="6"/>
+    <col min="8" max="8" width="12.140625" style="6" customWidth="1"/>
+    <col min="9" max="9" width="29.7109375" style="6" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
-      <c r="B1" s="5" t="s">
-        <v>3</v>
-      </c>
+      <c r="B1" s="5"/>
       <c r="H1" s="23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
       <c r="E2" s="24"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I3" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="17">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" s="25"/>
       <c r="H4" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+      <c r="I4" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="E5" s="27"/>
       <c r="H5" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+      <c r="I5" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
+      <c r="D6" s="22" t="s">
+        <v>32</v>
+      </c>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="14" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -817,7 +844,7 @@
       <c r="D10" s="1"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -826,7 +853,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
@@ -835,7 +862,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -844,7 +871,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -853,7 +880,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -862,7 +889,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -871,7 +898,7 @@
       <c r="D16" s="1"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -880,7 +907,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -889,7 +916,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -898,7 +925,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -907,7 +934,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -916,7 +943,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -925,7 +952,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -934,7 +961,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -943,7 +970,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -952,9 +979,9 @@
       <c r="D25" s="3"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C27" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="1"/>
@@ -979,79 +1006,89 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.26953125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="22.08984375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="4" width="16.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6"/>
+    <col min="9" max="9" width="22.140625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
-      <c r="B1" s="5" t="s">
-        <v>3</v>
-      </c>
+      <c r="B1" s="5"/>
       <c r="H1" s="23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
       <c r="E2" s="24"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I3" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="17">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E4" s="28"/>
       <c r="H4" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+      <c r="I4" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E5" s="30"/>
       <c r="H5" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+      <c r="I5" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
@@ -1059,28 +1096,28 @@
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1088,7 +1125,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1097,7 +1134,7 @@
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
@@ -1106,7 +1143,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1115,7 +1152,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1124,7 +1161,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1133,7 +1170,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1142,7 +1179,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1151,7 +1188,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1160,7 +1197,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1169,7 +1206,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1178,7 +1215,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1187,7 +1224,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1196,7 +1233,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1205,7 +1242,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1214,7 +1251,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1223,7 +1260,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1232,9 +1269,9 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C28" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="1"/>
@@ -1259,80 +1296,90 @@
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.26953125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.453125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="26.7265625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.85546875" style="6"/>
+    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
-      <c r="B1" s="5" t="s">
-        <v>3</v>
-      </c>
+      <c r="B1" s="5"/>
       <c r="H1" s="23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
       <c r="E2" s="24"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I3" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="17">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E4" s="31"/>
       <c r="H4" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+      <c r="I4" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5" s="33"/>
       <c r="H5" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+      <c r="I5" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
@@ -1340,28 +1387,28 @@
       <c r="D6" s="22"/>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="22"/>
       <c r="E7" s="22"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1369,7 +1416,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1378,7 +1425,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
@@ -1387,7 +1434,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1396,7 +1443,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1405,7 +1452,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1414,7 +1461,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1423,7 +1470,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1432,7 +1479,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1441,7 +1488,7 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1450,7 +1497,7 @@
       <c r="D19" s="1"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1459,7 +1506,7 @@
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1468,7 +1515,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1477,7 +1524,7 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1486,7 +1533,7 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1495,7 +1542,7 @@
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1504,7 +1551,7 @@
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1513,7 +1560,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1522,7 +1569,7 @@
       <c r="D27" s="2"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1531,7 +1578,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1540,7 +1587,7 @@
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1549,9 +1596,9 @@
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C32" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="1"/>
@@ -1576,77 +1623,87 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="6"/>
-    <col min="2" max="2" width="12.26953125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.26953125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="6"/>
+    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.90625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.6328125" style="6" customWidth="1"/>
-    <col min="7" max="8" width="8.90625" style="6"/>
-    <col min="9" max="9" width="26.7265625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.90625" style="6"/>
+    <col min="5" max="5" width="23.85546875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="6" customWidth="1"/>
+    <col min="7" max="8" width="8.85546875" style="6"/>
+    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
-      <c r="B1" s="5" t="s">
-        <v>3</v>
-      </c>
+      <c r="B1" s="5"/>
       <c r="H1" s="23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I1" s="23"/>
       <c r="J1" s="23"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
       <c r="E2" s="24"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I3" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="17">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="16" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D4" s="31"/>
       <c r="E4" s="31"/>
       <c r="H4" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+      <c r="I4" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="22"/>
       <c r="E5" s="22"/>
       <c r="H5" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+      <c r="I5" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>1</v>
@@ -1655,24 +1712,24 @@
       <c r="E6" s="22"/>
       <c r="F6" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D9" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1681,7 +1738,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1691,7 +1748,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
@@ -1701,7 +1758,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1711,7 +1768,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1721,7 +1778,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1731,7 +1788,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1741,7 +1798,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1751,7 +1808,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1761,7 +1818,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1771,7 +1828,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1781,7 +1838,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1791,7 +1848,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1801,7 +1858,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1811,7 +1868,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1821,7 +1878,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1831,7 +1888,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1841,7 +1898,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1851,7 +1908,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1861,7 +1918,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1871,7 +1928,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1881,15 +1938,15 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C32" s="34" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D32" s="35"/>
       <c r="E32" s="35"/>
       <c r="F32" s="18"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F35" s="21"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: finished requirements inspection
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moglan Calin-Stefan\CS UBB\SEM6\VVSS\MyDrinkShop\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F88C50A-6EA3-4AE1-AA21-0C13316182AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE12317-11AA-4499-8DB6-8A2AAA6FCC33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="3255" windowWidth="38700" windowHeight="15825" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26925" yWindow="3345" windowWidth="22620" windowHeight="15825" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="45">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -68,12 +68,6 @@
     <t xml:space="preserve">Author Name: </t>
   </si>
   <si>
-    <t>Popescu Ionel</t>
-  </si>
-  <si>
-    <t>Georgescu Anca</t>
-  </si>
-  <si>
     <t>Requirements Document</t>
   </si>
   <si>
@@ -141,6 +135,42 @@
   </si>
   <si>
     <t>Munteanu Valentin-Ioan</t>
+  </si>
+  <si>
+    <t>R01</t>
+  </si>
+  <si>
+    <t>R02</t>
+  </si>
+  <si>
+    <t>R04</t>
+  </si>
+  <si>
+    <t>R05</t>
+  </si>
+  <si>
+    <t>R07</t>
+  </si>
+  <si>
+    <t>Cerintele referitoare la actualizarea stocului nu specifica reactia aplicatiei in momentul in care cantitatea de ingrediente depaseste stocul disponibil</t>
+  </si>
+  <si>
+    <t>Nu se mentioneaza starea aplicatiei pentru prima rulare. Mai mult decat atat nu se specifica nimic despre existenta/necesitatea crearii fisierelor text in care se persista datele</t>
+  </si>
+  <si>
+    <t>Atributele produselor nu sunt specificate acestea fiind importante pentru calculul total al zilei. Pe langa asta nu ne este expus ce contine bonul generat in format .csv</t>
+  </si>
+  <si>
+    <t>15/03/2026</t>
+  </si>
+  <si>
+    <t>Sonar Qube</t>
+  </si>
+  <si>
+    <t>Se mentioneaza in cerinta faptul ca avem o aplicatie desktop Java - JavaFX, dar nu se specifica versiunea minima a JDK-ului necesara pentru rulare</t>
+  </si>
+  <si>
+    <t>Functia de export este definita ambiguu. Nu este clar ce exporta exact utilizatorul, ce informatii sunt exportate exact?</t>
   </si>
 </sst>
 </file>
@@ -339,7 +369,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -370,6 +400,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -412,7 +443,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -737,33 +768,33 @@
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
-      <c r="H1" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="H1" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="B2" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="36" t="s">
-        <v>31</v>
+        <v>16</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>29</v>
       </c>
       <c r="J3" s="17">
         <v>234</v>
@@ -773,15 +804,15 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="25"/>
+      <c r="D4" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="26"/>
       <c r="H4" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="36" t="s">
-        <v>33</v>
+        <v>17</v>
+      </c>
+      <c r="I4" s="22" t="s">
+        <v>31</v>
       </c>
       <c r="J4" s="3">
         <v>234</v>
@@ -791,15 +822,15 @@
       <c r="C5" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="27"/>
+      <c r="D5" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="28"/>
       <c r="H5" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="36" t="s">
-        <v>34</v>
+        <v>18</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>32</v>
       </c>
       <c r="J5" s="3">
         <v>234</v>
@@ -810,17 +841,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" s="22"/>
+      <c r="D6" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
+      <c r="D7" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="23"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -836,49 +869,69 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E10" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E11" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E12" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E13" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="D14" s="1"/>
-      <c r="E14" s="2"/>
+      <c r="E14" s="2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
@@ -984,7 +1037,9 @@
         <v>7</v>
       </c>
       <c r="D27" s="12"/>
-      <c r="E27" s="1"/>
+      <c r="E27" s="37">
+        <v>2.5694444444444443E-2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1020,33 +1075,33 @@
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
-      <c r="H1" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="H1" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="B2" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="36" t="s">
-        <v>31</v>
+        <v>16</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>29</v>
       </c>
       <c r="J3" s="17">
         <v>234</v>
@@ -1056,15 +1111,15 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="28" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="28"/>
+      <c r="D4" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="29"/>
       <c r="H4" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="36" t="s">
-        <v>33</v>
+        <v>17</v>
+      </c>
+      <c r="I4" s="22" t="s">
+        <v>31</v>
       </c>
       <c r="J4" s="3">
         <v>234</v>
@@ -1074,15 +1129,15 @@
       <c r="C5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="30"/>
+      <c r="D5" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="31"/>
       <c r="H5" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="36" t="s">
-        <v>34</v>
+        <v>18</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>32</v>
       </c>
       <c r="J5" s="3">
         <v>234</v>
@@ -1093,15 +1148,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
+      <c r="D7" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="23"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1311,33 +1370,33 @@
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
-      <c r="H1" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="H1" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="B2" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="36" t="s">
-        <v>31</v>
+        <v>16</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>29</v>
       </c>
       <c r="J3" s="17">
         <v>234</v>
@@ -1347,15 +1406,15 @@
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="31"/>
+      <c r="D4" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="32"/>
       <c r="H4" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="36" t="s">
-        <v>33</v>
+        <v>17</v>
+      </c>
+      <c r="I4" s="22" t="s">
+        <v>31</v>
       </c>
       <c r="J4" s="3">
         <v>234</v>
@@ -1365,15 +1424,15 @@
       <c r="C5" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="33"/>
+      <c r="D5" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="34"/>
       <c r="H5" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="36" t="s">
-        <v>34</v>
+        <v>18</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>32</v>
       </c>
       <c r="J5" s="3">
         <v>234</v>
@@ -1384,15 +1443,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
+      <c r="D7" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="23"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1639,33 +1702,33 @@
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
-      <c r="H1" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
+      <c r="H1" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="B2" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H3" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="36" t="s">
-        <v>31</v>
+        <v>16</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>29</v>
       </c>
       <c r="J3" s="17">
         <v>234</v>
@@ -1673,15 +1736,17 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C4" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+        <v>21</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="32"/>
       <c r="H4" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4" s="36" t="s">
-        <v>33</v>
+        <v>17</v>
+      </c>
+      <c r="I4" s="22" t="s">
+        <v>31</v>
       </c>
       <c r="J4" s="3">
         <v>234</v>
@@ -1691,13 +1756,15 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
+      <c r="D5" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="23"/>
       <c r="H5" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="36" t="s">
-        <v>34</v>
+        <v>18</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>32</v>
       </c>
       <c r="J5" s="3">
         <v>234</v>
@@ -1708,8 +1775,10 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="23"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -1717,16 +1786,16 @@
         <v>3</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D9" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1939,11 +2008,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C32" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
+      <c r="C32" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
       <c r="F32" s="18"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: added Doc: line/page values to every Rxx
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moglan Calin-Stefan\CS UBB\SEM6\VVSS\MyDrinkShop\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE12317-11AA-4499-8DB6-8A2AAA6FCC33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E394185-C8FE-42F9-A48F-2EFBD6BBA22F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26925" yWindow="3345" windowWidth="22620" windowHeight="15825" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="21705" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="50">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -171,6 +171,21 @@
   </si>
   <si>
     <t>Functia de export este definita ambiguu. Nu este clar ce exporta exact utilizatorul, ce informatii sunt exportate exact?</t>
+  </si>
+  <si>
+    <t>Cerinte Functionale - Cerinta 5</t>
+  </si>
+  <si>
+    <t>Cerinte Non-Functionale - Cerinta 1</t>
+  </si>
+  <si>
+    <t>Al doilea paragraf  - Linia 2</t>
+  </si>
+  <si>
+    <t>Cerinte Functionale - Cerinta 1</t>
+  </si>
+  <si>
+    <t>Cerinte Functionale - Cerinta 8</t>
   </si>
 </sst>
 </file>
@@ -369,7 +384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -401,6 +416,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -443,7 +459,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="20" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -768,19 +786,19 @@
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>26</v>
@@ -804,10 +822,10 @@
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="26"/>
+      <c r="E4" s="27"/>
       <c r="H4" s="17" t="s">
         <v>17</v>
       </c>
@@ -822,10 +840,10 @@
       <c r="C5" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="28"/>
+      <c r="E5" s="29"/>
       <c r="H5" s="17" t="s">
         <v>18</v>
       </c>
@@ -841,19 +859,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="23"/>
+      <c r="E6" s="24"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="23"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -876,7 +894,9 @@
       <c r="C10" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="1"/>
+      <c r="D10" s="38" t="s">
+        <v>45</v>
+      </c>
       <c r="E10" s="2" t="s">
         <v>38</v>
       </c>
@@ -889,7 +909,9 @@
       <c r="C11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="1"/>
+      <c r="D11" s="38" t="s">
+        <v>47</v>
+      </c>
       <c r="E11" s="2" t="s">
         <v>39</v>
       </c>
@@ -902,7 +924,9 @@
       <c r="C12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="1"/>
+      <c r="D12" s="38" t="s">
+        <v>48</v>
+      </c>
       <c r="E12" s="2" t="s">
         <v>40</v>
       </c>
@@ -915,7 +939,9 @@
       <c r="C13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="1"/>
+      <c r="D13" s="38" t="s">
+        <v>46</v>
+      </c>
       <c r="E13" s="2" t="s">
         <v>43</v>
       </c>
@@ -928,7 +954,9 @@
       <c r="C14" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="1"/>
+      <c r="D14" s="38" t="s">
+        <v>49</v>
+      </c>
       <c r="E14" s="2" t="s">
         <v>44</v>
       </c>
@@ -1037,7 +1065,7 @@
         <v>7</v>
       </c>
       <c r="D27" s="12"/>
-      <c r="E27" s="37">
+      <c r="E27" s="23">
         <v>2.5694444444444443E-2</v>
       </c>
     </row>
@@ -1075,19 +1103,19 @@
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>26</v>
@@ -1111,10 +1139,10 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="30"/>
       <c r="H4" s="17" t="s">
         <v>17</v>
       </c>
@@ -1129,10 +1157,10 @@
       <c r="C5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="31"/>
+      <c r="E5" s="32"/>
       <c r="H5" s="17" t="s">
         <v>18</v>
       </c>
@@ -1148,19 +1176,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="23"/>
+      <c r="E6" s="24"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="23"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1370,19 +1398,19 @@
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>26</v>
@@ -1406,10 +1434,10 @@
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>17</v>
       </c>
@@ -1424,10 +1452,10 @@
       <c r="C5" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="34"/>
+      <c r="E5" s="35"/>
       <c r="H5" s="17" t="s">
         <v>18</v>
       </c>
@@ -1443,19 +1471,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="23"/>
+      <c r="E6" s="24"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="23"/>
+      <c r="E7" s="24"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
@@ -1702,19 +1730,19 @@
     <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5"/>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>26</v>
@@ -1738,10 +1766,10 @@
       <c r="C4" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>17</v>
       </c>
@@ -1756,10 +1784,10 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="23"/>
+      <c r="E5" s="24"/>
       <c r="H5" s="17" t="s">
         <v>18</v>
       </c>
@@ -1775,10 +1803,10 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="23"/>
+      <c r="E6" s="24"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -2008,11 +2036,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C32" s="35" t="s">
+      <c r="C32" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
       <c r="F32" s="18"/>
     </row>
     <row r="35" spans="6:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: add inspection duration
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="58">
   <si>
     <t xml:space="preserve">Echipa</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t xml:space="preserve">Bad aggregation between FileOrderRepository and the Repository interface</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35 min</t>
   </si>
   <si>
     <t xml:space="preserve">Review Form. Coding Defects</t>
@@ -369,119 +372,119 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1351,7 +1354,9 @@
         <v>36</v>
       </c>
       <c r="D28" s="20"/>
-      <c r="E28" s="15"/>
+      <c r="E28" s="15" t="s">
+        <v>47</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1387,7 +1392,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.43"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.7"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.86"/>
   </cols>
   <sheetData>
@@ -1402,7 +1407,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1431,7 +1436,7 @@
         <v>6</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E4" s="26"/>
       <c r="H4" s="6" t="s">
@@ -1725,7 +1730,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.57"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="8.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.7"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="8.86"/>
   </cols>
   <sheetData>
@@ -1740,7 +1745,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1766,10 +1771,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C4" s="25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E4" s="26"/>
       <c r="H4" s="6" t="s">
@@ -1815,16 +1820,16 @@
         <v>17</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2038,7 +2043,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C32" s="28" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D32" s="28"/>
       <c r="E32" s="28"/>

</xml_diff>